<commit_message>
redo analysis without ex species
</commit_message>
<xml_diff>
--- a/builds/eradication_programs/sum_erad_tables.xlsx
+++ b/builds/eradication_programs/sum_erad_tables.xlsx
@@ -11,10 +11,8 @@
     <sheet name="sum_per_rodent" sheetId="2" r:id="rId2"/>
     <sheet name="sum_erad_status" sheetId="3" r:id="rId3"/>
     <sheet name="sum_per_rodent_erad_status" sheetId="4" r:id="rId4"/>
-    <sheet name="sum_extant" sheetId="5" r:id="rId5"/>
-    <sheet name="sum_per_rodent_extant" sheetId="6" r:id="rId6"/>
-    <sheet name="sum_extant_no_sing_end" sheetId="7" r:id="rId7"/>
-    <sheet name="sum_per_rodent_extant_no_sing" sheetId="8" r:id="rId8"/>
+    <sheet name="sum__no_sing_end" sheetId="5" r:id="rId5"/>
+    <sheet name="sum_per_rodent_no_sing_end" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -385,10 +383,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C2">
-        <v>39.38</v>
+        <v>40.31</v>
       </c>
     </row>
     <row r="3">
@@ -398,10 +396,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="C3">
-        <v>14.58</v>
+        <v>12.11</v>
       </c>
     </row>
     <row r="4">
@@ -414,7 +412,7 @@
         <v>26</v>
       </c>
       <c r="C4">
-        <v>5.42</v>
+        <v>5.73</v>
       </c>
     </row>
     <row r="5">
@@ -424,10 +422,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C5">
-        <v>21.67</v>
+        <v>21.81</v>
       </c>
     </row>
     <row r="6">
@@ -440,7 +438,7 @@
         <v>54</v>
       </c>
       <c r="C6">
-        <v>11.25</v>
+        <v>11.89</v>
       </c>
     </row>
     <row r="7">
@@ -453,7 +451,7 @@
         <v>37</v>
       </c>
       <c r="C7">
-        <v>7.71</v>
+        <v>8.15</v>
       </c>
     </row>
   </sheetData>
@@ -500,10 +498,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2">
-        <v>44.15</v>
+        <v>45.05</v>
       </c>
     </row>
     <row r="3">
@@ -518,10 +516,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D3">
-        <v>70.3</v>
+        <v>82.34999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -536,10 +534,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D4">
-        <v>17.42</v>
+        <v>15.52</v>
       </c>
     </row>
     <row r="5">
@@ -563,7 +561,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -572,16 +570,16 @@
         </is>
       </c>
       <c r="C6">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="D6">
-        <v>19.8</v>
+        <v>23.63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -590,10 +588,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="D7">
-        <v>22.87</v>
+        <v>5.88</v>
       </c>
     </row>
     <row r="8">
@@ -611,7 +609,7 @@
         <v>7</v>
       </c>
       <c r="D8">
-        <v>3.93</v>
+        <v>4.02</v>
       </c>
     </row>
     <row r="9">
@@ -629,7 +627,7 @@
         <v>3</v>
       </c>
       <c r="D9">
-        <v>2.97</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="10">
@@ -647,7 +645,7 @@
         <v>14</v>
       </c>
       <c r="D10">
-        <v>7.45</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="11">
@@ -683,7 +681,7 @@
         <v>90</v>
       </c>
       <c r="D12">
-        <v>50.56</v>
+        <v>51.72</v>
       </c>
     </row>
     <row r="13">
@@ -698,10 +696,10 @@
         </is>
       </c>
       <c r="C13">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D13">
-        <v>7.45</v>
+        <v>4.95</v>
       </c>
     </row>
     <row r="14">
@@ -719,7 +717,7 @@
         <v>24</v>
       </c>
       <c r="D14">
-        <v>13.48</v>
+        <v>13.79</v>
       </c>
     </row>
     <row r="15">
@@ -737,7 +735,7 @@
         <v>25</v>
       </c>
       <c r="D15">
-        <v>13.3</v>
+        <v>13.74</v>
       </c>
     </row>
     <row r="16">
@@ -755,7 +753,7 @@
         <v>5</v>
       </c>
       <c r="D16">
-        <v>4.95</v>
+        <v>5.88</v>
       </c>
     </row>
     <row r="17">
@@ -773,7 +771,7 @@
         <v>2</v>
       </c>
       <c r="D17">
-        <v>1.98</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="18">
@@ -791,7 +789,7 @@
         <v>26</v>
       </c>
       <c r="D18">
-        <v>14.61</v>
+        <v>14.94</v>
       </c>
     </row>
     <row r="19">
@@ -809,7 +807,7 @@
         <v>9</v>
       </c>
       <c r="D19">
-        <v>4.79</v>
+        <v>4.95</v>
       </c>
     </row>
   </sheetData>
@@ -819,7 +817,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -856,10 +854,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D2">
-        <v>23.96</v>
+        <v>24.89</v>
       </c>
     </row>
     <row r="3">
@@ -874,10 +872,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="D3">
-        <v>7.92</v>
+        <v>5.73</v>
       </c>
     </row>
     <row r="4">
@@ -895,7 +893,7 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>1.67</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="5">
@@ -910,10 +908,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D5">
-        <v>13.12</v>
+        <v>13.44</v>
       </c>
     </row>
     <row r="6">
@@ -931,7 +929,7 @@
         <v>38</v>
       </c>
       <c r="D6">
-        <v>7.92</v>
+        <v>8.369999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -949,7 +947,7 @@
         <v>22</v>
       </c>
       <c r="D7">
-        <v>4.58</v>
+        <v>4.85</v>
       </c>
     </row>
     <row r="8">
@@ -964,10 +962,10 @@
         </is>
       </c>
       <c r="C8">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D8">
-        <v>7.92</v>
+        <v>7.71</v>
       </c>
     </row>
     <row r="9">
@@ -985,7 +983,7 @@
         <v>9</v>
       </c>
       <c r="D9">
-        <v>1.88</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="10">
@@ -1003,7 +1001,7 @@
         <v>3</v>
       </c>
       <c r="D10">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="11">
@@ -1018,10 +1016,10 @@
         </is>
       </c>
       <c r="C11">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D11">
-        <v>7.29</v>
+        <v>7.05</v>
       </c>
     </row>
     <row r="12">
@@ -1039,7 +1037,7 @@
         <v>6</v>
       </c>
       <c r="D12">
-        <v>1.25</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="13">
@@ -1057,7 +1055,7 @@
         <v>12</v>
       </c>
       <c r="D13">
-        <v>2.5</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="14">
@@ -1075,7 +1073,7 @@
         <v>10</v>
       </c>
       <c r="D14">
-        <v>2.08</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="15">
@@ -1090,10 +1088,10 @@
         </is>
       </c>
       <c r="C15">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D15">
-        <v>2.29</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="16">
@@ -1111,7 +1109,7 @@
         <v>10</v>
       </c>
       <c r="D16">
-        <v>2.08</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="17">
@@ -1129,7 +1127,7 @@
         <v>2</v>
       </c>
       <c r="D17">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="18">
@@ -1147,7 +1145,7 @@
         <v>5</v>
       </c>
       <c r="D18">
-        <v>1.04</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="19">
@@ -1165,7 +1163,7 @@
         <v>2</v>
       </c>
       <c r="D19">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="20">
@@ -1183,7 +1181,7 @@
         <v>3</v>
       </c>
       <c r="D20">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="21">
@@ -1201,7 +1199,7 @@
         <v>4</v>
       </c>
       <c r="D21">
-        <v>0.83</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="22">
@@ -1219,13 +1217,13 @@
         <v>3</v>
       </c>
       <c r="D22">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1237,13 +1235,13 @@
         <v>1</v>
       </c>
       <c r="D23">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Population study without data in support</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1255,13 +1253,13 @@
         <v>1</v>
       </c>
       <c r="D24">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Population study without data in support</t>
+          <t>Population study with data in support</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1273,31 +1271,31 @@
         <v>1</v>
       </c>
       <c r="D25">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Population study with data in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26">
-        <v>0.21</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1309,13 +1307,13 @@
         <v>2</v>
       </c>
       <c r="D27">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Only predation in support</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1324,16 +1322,16 @@
         </is>
       </c>
       <c r="C28">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D28">
-        <v>0.42</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Only predation in support</t>
+          <t>Population study without data in support</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1342,34 +1340,34 @@
         </is>
       </c>
       <c r="C29">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D29">
-        <v>1.04</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Population study without data in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="C30">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30">
-        <v>0.21</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>Population study without data in support</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1378,34 +1376,34 @@
         </is>
       </c>
       <c r="C31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31">
-        <v>0.62</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Population study without data in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Incomplete</t>
+          <t>Trial or Research only</t>
         </is>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D32">
-        <v>0.21</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1414,28 +1412,28 @@
         </is>
       </c>
       <c r="C33">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D33">
-        <v>2.5</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Trial or Research only</t>
+          <t>Unknown pre-status</t>
         </is>
       </c>
       <c r="C34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D34">
-        <v>0.62</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="35">
@@ -1446,20 +1444,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Unknown pre-status</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C35">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D35">
-        <v>0.83</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1468,16 +1466,16 @@
         </is>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36">
-        <v>0.42</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Population study without data in support</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1486,28 +1484,10 @@
         </is>
       </c>
       <c r="C37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37">
-        <v>0.62</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Population study without data in support</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C38">
-        <v>1</v>
-      </c>
-      <c r="D38">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
     </row>
   </sheetData>
@@ -1517,7 +1497,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1564,10 +1544,10 @@
         </is>
       </c>
       <c r="D2">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E2">
-        <v>57.43</v>
+        <v>67.06</v>
       </c>
     </row>
     <row r="3">
@@ -1590,7 +1570,7 @@
         <v>41</v>
       </c>
       <c r="E3">
-        <v>21.81</v>
+        <v>22.53</v>
       </c>
     </row>
     <row r="4">
@@ -1610,10 +1590,10 @@
         </is>
       </c>
       <c r="D4">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E4">
-        <v>6.74</v>
+        <v>6.32</v>
       </c>
     </row>
     <row r="5">
@@ -1642,7 +1622,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1656,16 +1636,16 @@
         </is>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E6">
-        <v>13.86</v>
+        <v>10.44</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1679,10 +1659,10 @@
         </is>
       </c>
       <c r="D7">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>10.11</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="8">
@@ -1705,7 +1685,7 @@
         <v>5</v>
       </c>
       <c r="E8">
-        <v>2.81</v>
+        <v>2.87</v>
       </c>
     </row>
     <row r="9">
@@ -1728,7 +1708,7 @@
         <v>5</v>
       </c>
       <c r="E9">
-        <v>2.66</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="10">
@@ -1774,7 +1754,7 @@
         <v>53</v>
       </c>
       <c r="E11">
-        <v>29.78</v>
+        <v>30.46</v>
       </c>
     </row>
     <row r="12">
@@ -1794,10 +1774,10 @@
         </is>
       </c>
       <c r="D12">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E12">
-        <v>5.32</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="13">
@@ -1820,7 +1800,7 @@
         <v>20</v>
       </c>
       <c r="E13">
-        <v>11.24</v>
+        <v>11.49</v>
       </c>
     </row>
     <row r="14">
@@ -1843,7 +1823,7 @@
         <v>4</v>
       </c>
       <c r="E14">
-        <v>3.96</v>
+        <v>4.71</v>
       </c>
     </row>
     <row r="15">
@@ -1866,7 +1846,7 @@
         <v>14</v>
       </c>
       <c r="E15">
-        <v>7.45</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="16">
@@ -1889,7 +1869,7 @@
         <v>2</v>
       </c>
       <c r="E16">
-        <v>1.98</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="17">
@@ -1912,7 +1892,7 @@
         <v>14</v>
       </c>
       <c r="E17">
-        <v>7.87</v>
+        <v>8.050000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -1935,7 +1915,7 @@
         <v>6</v>
       </c>
       <c r="E18">
-        <v>3.19</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="19">
@@ -1955,10 +1935,10 @@
         </is>
       </c>
       <c r="D19">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E19">
-        <v>14.89</v>
+        <v>14.84</v>
       </c>
     </row>
     <row r="20">
@@ -1978,10 +1958,10 @@
         </is>
       </c>
       <c r="D20">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E20">
-        <v>2.81</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="21">
@@ -2004,7 +1984,7 @@
         <v>5</v>
       </c>
       <c r="E21">
-        <v>4.95</v>
+        <v>5.88</v>
       </c>
     </row>
     <row r="22">
@@ -2027,7 +2007,7 @@
         <v>9</v>
       </c>
       <c r="E22">
-        <v>4.79</v>
+        <v>4.95</v>
       </c>
     </row>
     <row r="23">
@@ -2050,7 +2030,7 @@
         <v>3</v>
       </c>
       <c r="E23">
-        <v>1.6</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="24">
@@ -2073,7 +2053,7 @@
         <v>32</v>
       </c>
       <c r="E24">
-        <v>17.98</v>
+        <v>18.39</v>
       </c>
     </row>
     <row r="25">
@@ -2084,7 +2064,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Population study without data in support</t>
+          <t>Population study with data in support</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2093,16 +2073,16 @@
         </is>
       </c>
       <c r="D25">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E25">
-        <v>1.6</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus norvegicus</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2116,10 +2096,10 @@
         </is>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E26">
-        <v>2.66</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="27">
@@ -2130,7 +2110,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Population study with data in support</t>
+          <t>Population study with all qualities in support</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2139,16 +2119,16 @@
         </is>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E27">
-        <v>0.5600000000000001</v>
+        <v>5.17</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2162,10 +2142,10 @@
         </is>
       </c>
       <c r="D28">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E28">
-        <v>5.06</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="29">
@@ -2176,25 +2156,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Population study with all qualities in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Successful (Reinvaded)</t>
+          <t>Failed</t>
         </is>
       </c>
       <c r="D29">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E29">
-        <v>1.6</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2208,21 +2188,21 @@
         </is>
       </c>
       <c r="D30">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E30">
-        <v>3.19</v>
+        <v>4.71</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2231,16 +2211,16 @@
         </is>
       </c>
       <c r="D31">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E31">
-        <v>3.96</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2254,10 +2234,10 @@
         </is>
       </c>
       <c r="D32">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E32">
-        <v>3.72</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="33">
@@ -2268,7 +2248,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Only predation in support</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2277,16 +2257,16 @@
         </is>
       </c>
       <c r="D33">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33">
-        <v>3.96</v>
+        <v>3.53</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Mus musculus</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2300,16 +2280,16 @@
         </is>
       </c>
       <c r="D34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E34">
-        <v>2.97</v>
+        <v>15.38</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mus musculus</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2323,21 +2303,21 @@
         </is>
       </c>
       <c r="D35">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E35">
-        <v>15.38</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus norvegicus</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Only predation in support</t>
+          <t>Population study without data in support</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2346,10 +2326,10 @@
         </is>
       </c>
       <c r="D36">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E36">
-        <v>2.66</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="37">
@@ -2360,7 +2340,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Population study without data in support</t>
+          <t>Population study with data in support</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2369,16 +2349,16 @@
         </is>
       </c>
       <c r="D37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E37">
-        <v>1.12</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2392,16 +2372,16 @@
         </is>
       </c>
       <c r="D38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E38">
-        <v>1.69</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2418,41 +2398,41 @@
         <v>1</v>
       </c>
       <c r="E39">
-        <v>0.99</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Population study with data in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>To Be Confirmed</t>
         </is>
       </c>
       <c r="D40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40">
-        <v>0.53</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2464,13 +2444,13 @@
         <v>2</v>
       </c>
       <c r="E41">
-        <v>1.98</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2484,21 +2464,21 @@
         </is>
       </c>
       <c r="D42">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42">
-        <v>1.06</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Population study with data in support</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2507,21 +2487,21 @@
         </is>
       </c>
       <c r="D43">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E43">
-        <v>0.99</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus norvegicus</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Population study with data in support</t>
+          <t>Population study with all qualities in support</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2530,10 +2510,10 @@
         </is>
       </c>
       <c r="D44">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44">
-        <v>2.13</v>
+        <v>1.72</v>
       </c>
     </row>
     <row r="45">
@@ -2544,19 +2524,19 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Population study with all qualities in support</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>To Be Confirmed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="D45">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E45">
-        <v>1.69</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="46">
@@ -2567,7 +2547,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>Population study without data in support</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2579,18 +2559,18 @@
         <v>1</v>
       </c>
       <c r="E46">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Population study with data in support</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2602,53 +2582,53 @@
         <v>1</v>
       </c>
       <c r="E47">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Population study without data in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D48">
         <v>1</v>
       </c>
       <c r="E48">
-        <v>0.5600000000000001</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus norvegicus</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Population study with data in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D49">
         <v>1</v>
       </c>
       <c r="E49">
-        <v>0.53</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="50">
@@ -2659,7 +2639,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2671,18 +2651,18 @@
         <v>1</v>
       </c>
       <c r="E50">
-        <v>0.99</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2694,18 +2674,18 @@
         <v>1</v>
       </c>
       <c r="E51">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Mus musculus</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Only predation in support</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2714,10 +2694,10 @@
         </is>
       </c>
       <c r="D52">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E52">
-        <v>0.99</v>
+        <v>30.77</v>
       </c>
     </row>
     <row r="53">
@@ -2728,7 +2708,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Only predation in support</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2740,18 +2720,18 @@
         <v>1</v>
       </c>
       <c r="E53">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Mus musculus</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Only predation in support</t>
+          <t>Population study without data in support</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2760,10 +2740,10 @@
         </is>
       </c>
       <c r="D54">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E54">
-        <v>30.77</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="55">
@@ -2774,25 +2754,25 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Only predation in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="D55">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E55">
-        <v>0.53</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus norvegicus</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2802,20 +2782,20 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="D56">
         <v>1</v>
       </c>
       <c r="E56">
-        <v>0.53</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus norvegicus</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2825,43 +2805,43 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Incomplete</t>
+          <t>Trial or Research only</t>
         </is>
       </c>
       <c r="D57">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E57">
-        <v>1.6</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Population study without data in support</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Incomplete</t>
+          <t>Trial or Research only</t>
         </is>
       </c>
       <c r="D58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E58">
-        <v>0.5600000000000001</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Rattus norvegicus</t>
+          <t>Rattus rattus</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2871,14 +2851,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Trial or Research only</t>
+          <t>Unknown pre-status</t>
         </is>
       </c>
       <c r="D59">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E59">
-        <v>6.74</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="60">
@@ -2889,25 +2869,25 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>No studies found</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Trial or Research only</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E60">
-        <v>1.6</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus exulans</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2917,14 +2897,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Unknown pre-status</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D61">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E61">
-        <v>2.13</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="62">
@@ -2935,7 +2915,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2944,21 +2924,21 @@
         </is>
       </c>
       <c r="D62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62">
-        <v>0.53</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Rattus exulans</t>
+          <t>Rattus norvegicus</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>No studies found</t>
+          <t>All studies are not in support</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2970,18 +2950,18 @@
         <v>1</v>
       </c>
       <c r="E63">
-        <v>0.99</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Rattus rattus</t>
+          <t>Rattus norvegicus</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>All studies are not in support</t>
+          <t>Population study without data in support</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2990,56 +2970,10 @@
         </is>
       </c>
       <c r="D64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E64">
-        <v>1.06</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Rattus norvegicus</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>All studies are not in support</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="D65">
-        <v>1</v>
-      </c>
-      <c r="E65">
-        <v>0.5600000000000001</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Rattus norvegicus</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Population study without data in support</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="D66">
-        <v>1</v>
-      </c>
-      <c r="E66">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
     </row>
   </sheetData>
@@ -3076,10 +3010,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C2">
-        <v>40.31</v>
+        <v>40.35</v>
       </c>
     </row>
     <row r="3">
@@ -3092,7 +3026,7 @@
         <v>55</v>
       </c>
       <c r="C3">
-        <v>12.11</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="4">
@@ -3102,10 +3036,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4">
-        <v>5.73</v>
+        <v>5.32</v>
       </c>
     </row>
     <row r="5">
@@ -3118,7 +3052,7 @@
         <v>99</v>
       </c>
       <c r="C5">
-        <v>21.81</v>
+        <v>21.95</v>
       </c>
     </row>
     <row r="6">
@@ -3131,7 +3065,7 @@
         <v>54</v>
       </c>
       <c r="C6">
-        <v>11.89</v>
+        <v>11.97</v>
       </c>
     </row>
     <row r="7">
@@ -3144,7 +3078,7 @@
         <v>37</v>
       </c>
       <c r="C7">
-        <v>8.15</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3194,467 +3128,6 @@
         <v>82</v>
       </c>
       <c r="D2">
-        <v>45.05</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Rattus exulans</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>No studies found</t>
-        </is>
-      </c>
-      <c r="C3">
-        <v>70</v>
-      </c>
-      <c r="D3">
-        <v>82.34999999999999</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Rattus norvegicus</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>No studies found</t>
-        </is>
-      </c>
-      <c r="C4">
-        <v>27</v>
-      </c>
-      <c r="D4">
-        <v>15.52</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Mus musculus</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>No studies found</t>
-        </is>
-      </c>
-      <c r="C5">
-        <v>4</v>
-      </c>
-      <c r="D5">
-        <v>30.77</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Rattus rattus</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>All studies are not in support</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>43</v>
-      </c>
-      <c r="D6">
-        <v>23.63</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Rattus exulans</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>All studies are not in support</t>
-        </is>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-      <c r="D7">
-        <v>5.88</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Rattus norvegicus</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>All studies are not in support</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>7</v>
-      </c>
-      <c r="D8">
-        <v>4.02</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Rattus exulans</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Only predation in support</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>3</v>
-      </c>
-      <c r="D9">
-        <v>3.53</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Rattus rattus</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Only predation in support</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>14</v>
-      </c>
-      <c r="D10">
-        <v>7.69</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Mus musculus</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Only predation in support</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>9</v>
-      </c>
-      <c r="D11">
-        <v>69.23</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Rattus norvegicus</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Population study without data in support</t>
-        </is>
-      </c>
-      <c r="C12">
-        <v>90</v>
-      </c>
-      <c r="D12">
-        <v>51.72</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Rattus rattus</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Population study without data in support</t>
-        </is>
-      </c>
-      <c r="C13">
-        <v>9</v>
-      </c>
-      <c r="D13">
-        <v>4.95</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Rattus norvegicus</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Population study with data in support</t>
-        </is>
-      </c>
-      <c r="C14">
-        <v>24</v>
-      </c>
-      <c r="D14">
-        <v>13.79</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Rattus rattus</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Population study with data in support</t>
-        </is>
-      </c>
-      <c r="C15">
-        <v>25</v>
-      </c>
-      <c r="D15">
-        <v>13.74</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Rattus exulans</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Population study with data in support</t>
-        </is>
-      </c>
-      <c r="C16">
-        <v>5</v>
-      </c>
-      <c r="D16">
-        <v>5.88</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Rattus exulans</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Population study with all qualities in support</t>
-        </is>
-      </c>
-      <c r="C17">
-        <v>2</v>
-      </c>
-      <c r="D17">
-        <v>2.35</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Rattus norvegicus</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Population study with all qualities in support</t>
-        </is>
-      </c>
-      <c r="C18">
-        <v>26</v>
-      </c>
-      <c r="D18">
-        <v>14.94</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Rattus rattus</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Population study with all qualities in support</t>
-        </is>
-      </c>
-      <c r="C19">
-        <v>9</v>
-      </c>
-      <c r="D19">
-        <v>4.95</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Proportion</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No studies found</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>182</v>
-      </c>
-      <c r="C2">
-        <v>40.35</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>All studies are not in support</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>55</v>
-      </c>
-      <c r="C3">
-        <v>12.2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Only predation in support</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>24</v>
-      </c>
-      <c r="C4">
-        <v>5.32</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Population study without data in support</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>99</v>
-      </c>
-      <c r="C5">
-        <v>21.95</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Population study with data in support</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>54</v>
-      </c>
-      <c r="C6">
-        <v>11.97</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Population study with all qualities in support</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>37</v>
-      </c>
-      <c r="C7">
-        <v>8.199999999999999</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Rodent attributed</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Proportion</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Rattus rattus</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>No studies found</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>82</v>
-      </c>
-      <c r="D2">
         <v>45.56</v>
       </c>
     </row>

</xml_diff>